<commit_message>
Date and time is properly retrieved and stored into Transaction attributes
</commit_message>
<xml_diff>
--- a/Capstone 1 ToDo.xlsx
+++ b/Capstone 1 ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fernando\pluralsight\capstones\accounting-ledger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991429AA-81B1-4EBA-9B0C-14B0B8A2793D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586EE5CE-45E2-4586-BE26-7F6212894351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30840" yWindow="2040" windowWidth="21600" windowHeight="11385" xr2:uid="{ADEF4EBA-F5D9-4B5F-8B0D-DFDA391BE8B3}"/>
+    <workbookView xWindow="30465" yWindow="3255" windowWidth="21600" windowHeight="11385" xr2:uid="{ADEF4EBA-F5D9-4B5F-8B0D-DFDA391BE8B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -138,7 +138,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,6 +150,13 @@
       <b/>
       <sz val="20"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -187,13 +194,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,6 +571,7 @@
       <c r="B3" t="s">
         <v>20</v>
       </c>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -571,11 +580,13 @@
       <c r="B4" t="s">
         <v>20</v>
       </c>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -605,6 +616,7 @@
       <c r="B10" t="s">
         <v>28</v>
       </c>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -613,6 +625,7 @@
       <c r="B11" t="s">
         <v>29</v>
       </c>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">

</xml_diff>

<commit_message>
Ledger displays all entries from previous year
</commit_message>
<xml_diff>
--- a/Capstone 1 ToDo.xlsx
+++ b/Capstone 1 ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fernando\pluralsight\capstones\accounting-ledger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586EE5CE-45E2-4586-BE26-7F6212894351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE0605D-250D-40B9-BC37-A3BD9356304E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30465" yWindow="3255" windowWidth="21600" windowHeight="11385" xr2:uid="{ADEF4EBA-F5D9-4B5F-8B0D-DFDA391BE8B3}"/>
+    <workbookView xWindow="30465" yWindow="2670" windowWidth="21600" windowHeight="11970" xr2:uid="{ADEF4EBA-F5D9-4B5F-8B0D-DFDA391BE8B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -594,6 +594,9 @@
       </c>
       <c r="C6" s="2"/>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="2"/>
+    </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
@@ -631,11 +634,16 @@
       <c r="A12" t="s">
         <v>21</v>
       </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -644,6 +652,7 @@
       <c r="B15" t="s">
         <v>23</v>
       </c>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -653,36 +662,42 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>12</v>
       </c>
       <c r="B17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>14</v>
       </c>
       <c r="B19" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>

</xml_diff>